<commit_message>
[fix/HD-845-usage-stats-report] added difference explaining legend
</commit_message>
<xml_diff>
--- a/api/templates/usage_statistics_report/en.xlsx
+++ b/api/templates/usage_statistics_report/en.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\usage_statistics_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6B1812-DB3E-4EAF-BEAC-C60C38ECA2BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB1FE40-3E7F-43FF-8E16-E6EBE7270455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
   <si>
     <t>&lt;StatesLabel&gt;:  &lt;States&gt;</t>
   </si>
@@ -122,6 +122,9 @@
   </si>
   <si>
     <t>Dates:  &lt;Dates&gt;</t>
+  </si>
+  <si>
+    <t>* You may notice small differences in quantities of devices and results between this report and on screen lists. This is because in order to show the reported results versus performed results, this report is considering the date of creation of the result, instead of the date of completion.</t>
   </si>
 </sst>
 </file>
@@ -312,7 +315,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -346,6 +349,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -745,7 +751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="38.109375" bestFit="1" customWidth="1"/>
@@ -757,38 +763,38 @@
     <col min="7" max="7" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>27</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="2"/>
     </row>
-    <row r="7" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="1:2" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:4" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>5</v>
       </c>
@@ -796,7 +802,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>6</v>
       </c>
@@ -804,7 +810,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -812,7 +818,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
@@ -820,7 +826,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>9</v>
       </c>
@@ -828,7 +834,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>10</v>
       </c>
@@ -836,11 +842,46 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14"/>
       <c r="B14" s="13"/>
     </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A15:D19"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
#ASP-6999 Show page view in usage statistics
</commit_message>
<xml_diff>
--- a/api/templates/usage_statistics_report/en.xlsx
+++ b/api/templates/usage_statistics_report/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10912"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\usage_statistics_report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mehdi/Desktop/Projects/SystemOne/aspect/api/templates/usage_statistics_report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB1FE40-3E7F-43FF-8E16-E6EBE7270455}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26C88043-4A1A-A24F-8F50-1B1D87F8893C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17400" yWindow="700" windowWidth="34000" windowHeight="25680" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Usage Totals" sheetId="1" r:id="rId1"/>
@@ -25,12 +25,8 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
   <si>
     <t>&lt;StatesLabel&gt;:  &lt;States&gt;</t>
   </si>
@@ -125,6 +121,12 @@
   </si>
   <si>
     <t>* You may notice small differences in quantities of devices and results between this report and on screen lists. This is because in order to show the reported results versus performed results, this report is considering the date of creation of the result, instead of the date of completion.</t>
+  </si>
+  <si>
+    <t>Page Views</t>
+  </si>
+  <si>
+    <t>&lt;pageView&gt;</t>
   </si>
 </sst>
 </file>
@@ -752,49 +754,49 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D19"/>
-  <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="38.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.6640625" customWidth="1"/>
-    <col min="3" max="3" width="18.77734375" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" customWidth="1"/>
-    <col min="5" max="5" width="16.44140625" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.5" customWidth="1"/>
+    <col min="5" max="5" width="16.5" customWidth="1"/>
     <col min="6" max="6" width="21" customWidth="1"/>
     <col min="7" max="7" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="2"/>
     </row>
-    <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
       <c r="B4" s="2"/>
     </row>
-    <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="2"/>
     </row>
-    <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="8" spans="1:4" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="1:4" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A8" s="10" t="s">
         <v>5</v>
       </c>
@@ -802,7 +804,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
         <v>6</v>
       </c>
@@ -810,7 +812,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>7</v>
       </c>
@@ -818,7 +820,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>8</v>
       </c>
@@ -826,7 +828,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>9</v>
       </c>
@@ -834,7 +836,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>10</v>
       </c>
@@ -842,11 +844,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="16.2" thickTop="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A14" s="14"/>
       <c r="B14" s="13"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="15" t="s">
         <v>28</v>
       </c>
@@ -854,25 +856,25 @@
       <c r="C15" s="15"/>
       <c r="D15" s="15"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="15"/>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="15"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="15"/>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
       <c r="D17" s="15"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="15"/>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="15"/>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -889,42 +891,49 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40AC2301-C80C-4FC7-B9AE-64396E099A82}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="30.77734375" customWidth="1"/>
-    <col min="2" max="2" width="27.77734375" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="27.83203125" customWidth="1"/>
+    <col min="3" max="3" width="27.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>22</v>
       </c>
       <c r="B6" t="s">
         <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -935,42 +944,42 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ABE005F9-733A-4A93-ADFC-E0BBDF628800}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="3" width="22.88671875" customWidth="1"/>
+    <col min="1" max="3" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
         <v>18</v>
       </c>
@@ -981,7 +990,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>23</v>
       </c>

</xml_diff>